<commit_message>
diagnosis for no rule fire fixed
</commit_message>
<xml_diff>
--- a/backup/rules_2.xlsx
+++ b/backup/rules_2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="148">
   <si>
     <t>RuleSet</t>
   </si>
@@ -40,7 +40,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Agenda</t>
+    <t>AGENDA-GROUP</t>
   </si>
   <si>
     <t>Condition</t>
@@ -55,12 +55,6 @@
     <t>$s</t>
   </si>
   <si>
-    <t>getString("/account/statusFrom") == "$1"</t>
-  </si>
-  <si>
-    <t>getString("/account/statusTo") == "$1"</t>
-  </si>
-  <si>
     <t>getString("/account/equityOpenPosition") == "$1"</t>
   </si>
   <si>
@@ -154,12 +148,6 @@
     <t>set("/account/output/statusTo", "$param");</t>
   </si>
   <si>
-    <t>/account/statusFrom</t>
-  </si>
-  <si>
-    <t>/account/statusTo</t>
-  </si>
-  <si>
     <t>/account/equityOpenPosition</t>
   </si>
   <si>
@@ -334,12 +322,6 @@
     <t>Primary DP must be $expected but found $actual</t>
   </si>
   <si>
-    <t>Initial Status</t>
-  </si>
-  <si>
-    <t>Expected Status</t>
-  </si>
-  <si>
     <t>EquityPosn</t>
   </si>
   <si>
@@ -433,34 +415,46 @@
     <t>Status</t>
   </si>
   <si>
-    <t>activeToSelllingOnly1</t>
-  </si>
-  <si>
-    <t>activeToSellingOnly</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>SO</t>
+    <t>activeToFreezeR</t>
+  </si>
+  <si>
+    <t>"activeToFreeze"</t>
   </si>
   <si>
     <t>N</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>ALLOWED</t>
   </si>
   <si>
+    <t>FREEZE</t>
+  </si>
+  <si>
+    <t>activeToSelllingOnlyR</t>
+  </si>
+  <si>
+    <t>"activeToSellingOnly"</t>
+  </si>
+  <si>
     <t>SELLING ONLY</t>
   </si>
   <si>
-    <t>activeToSelllingOnly2</t>
-  </si>
-  <si>
-    <t>activeToSelllingOnly3</t>
+    <t>activeToInactiveR</t>
+  </si>
+  <si>
+    <t>"activeToInactive"</t>
+  </si>
+  <si>
+    <t>INACTIVE</t>
+  </si>
+  <si>
+    <t>activeToBuyingOnlyR</t>
+  </si>
+  <si>
+    <t>"activeToBuyingOnly"</t>
+  </si>
+  <si>
+    <t>BUYING ONLY</t>
   </si>
 </sst>
 </file>
@@ -488,7 +482,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color indexed="12"/>
+      <color indexed="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -498,7 +492,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -508,12 +502,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="9"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="10"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -544,7 +532,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="14"/>
+        <fgColor indexed="15"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -563,7 +551,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="15"/>
+        <fgColor indexed="16"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -585,8 +573,20 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="20"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="21"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -615,6 +615,128 @@
       </left>
       <right/>
       <top style="thin">
+        <color indexed="12"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="12"/>
+      </right>
+      <top style="thin">
+        <color indexed="12"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="12"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="12"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="14"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="14"/>
+      </left>
+      <right style="thin">
+        <color indexed="14"/>
+      </right>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="14"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right/>
+      <top style="thin">
         <color indexed="11"/>
       </top>
       <bottom style="thin">
@@ -625,10 +747,25 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="16"/>
+        <color indexed="12"/>
       </right>
       <top style="thin">
         <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="14"/>
       </top>
       <bottom style="thin">
         <color indexed="11"/>
@@ -652,29 +789,47 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="6" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -683,16 +838,28 @@
     <xf numFmtId="49" fontId="4" fillId="7" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="8" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -704,13 +871,19 @@
     <xf numFmtId="49" fontId="0" fillId="11" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="12" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="12" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="12" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="12" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="13" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="13" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="13" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -734,13 +907,15 @@
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
       <rgbColor rgb="ffe3e6e4"/>
+      <rgbColor rgb="ffffffff"/>
+      <rgbColor rgb="ffa5a5a5"/>
+      <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="ffffc000"/>
+      <rgbColor rgb="ffbbbbbb"/>
+      <rgbColor rgb="fff19d64"/>
       <rgbColor rgb="ffd2d2d2"/>
-      <rgbColor rgb="ffa5a5a5"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffffc000"/>
-      <rgbColor rgb="fff19d64"/>
       <rgbColor rgb="ff93c175"/>
-      <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="ffdddddd"/>
       <rgbColor rgb="fff19d64"/>
       <rgbColor rgb="ffb7d6a3"/>
       <rgbColor rgb="ffadcdea"/>
@@ -1778,1151 +1953,1159 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AI15"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="2" width="28.6719" style="1" customWidth="1"/>
-    <col min="3" max="5" width="45.6719" style="1" customWidth="1"/>
-    <col min="6" max="6" width="47.6719" style="1" customWidth="1"/>
-    <col min="7" max="9" width="45.6719" style="1" customWidth="1"/>
-    <col min="10" max="10" width="47.3516" style="1" customWidth="1"/>
-    <col min="11" max="11" width="50.1719" style="1" customWidth="1"/>
-    <col min="12" max="12" width="53.3672" style="1" customWidth="1"/>
-    <col min="13" max="13" width="60.5" style="1" customWidth="1"/>
-    <col min="14" max="14" width="54.5" style="1" customWidth="1"/>
-    <col min="15" max="15" width="62" style="1" customWidth="1"/>
-    <col min="16" max="16" width="63.6719" style="1" customWidth="1"/>
-    <col min="17" max="17" width="56.6719" style="1" customWidth="1"/>
-    <col min="18" max="18" width="59" style="1" customWidth="1"/>
-    <col min="19" max="19" width="64.6719" style="1" customWidth="1"/>
-    <col min="20" max="20" width="73.7266" style="1" customWidth="1"/>
-    <col min="21" max="21" width="68.8516" style="1" customWidth="1"/>
-    <col min="22" max="22" width="56.1719" style="1" customWidth="1"/>
-    <col min="23" max="23" width="65.1719" style="1" customWidth="1"/>
-    <col min="24" max="31" width="49.2656" style="1" customWidth="1"/>
-    <col min="32" max="32" width="52.5" style="1" customWidth="1"/>
-    <col min="33" max="33" width="49.2656" style="1" customWidth="1"/>
-    <col min="34" max="35" width="40.1719" style="1" customWidth="1"/>
-    <col min="36" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col min="3" max="4" width="45.6719" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47.6719" style="1" customWidth="1"/>
+    <col min="6" max="8" width="45.6719" style="1" customWidth="1"/>
+    <col min="9" max="9" width="47.3516" style="1" customWidth="1"/>
+    <col min="10" max="10" width="50.1719" style="1" customWidth="1"/>
+    <col min="11" max="11" width="53.3672" style="1" customWidth="1"/>
+    <col min="12" max="12" width="60.5" style="1" customWidth="1"/>
+    <col min="13" max="13" width="54.5" style="1" customWidth="1"/>
+    <col min="14" max="14" width="62" style="1" customWidth="1"/>
+    <col min="15" max="15" width="63.6719" style="1" customWidth="1"/>
+    <col min="16" max="16" width="56.6719" style="1" customWidth="1"/>
+    <col min="17" max="17" width="59" style="1" customWidth="1"/>
+    <col min="18" max="18" width="64.6719" style="1" customWidth="1"/>
+    <col min="19" max="19" width="73.7266" style="1" customWidth="1"/>
+    <col min="20" max="20" width="68.8516" style="1" customWidth="1"/>
+    <col min="21" max="21" width="56.1719" style="1" customWidth="1"/>
+    <col min="22" max="22" width="65.1719" style="1" customWidth="1"/>
+    <col min="23" max="30" width="49.2656" style="1" customWidth="1"/>
+    <col min="31" max="31" width="52.5" style="1" customWidth="1"/>
+    <col min="32" max="32" width="49.2656" style="1" customWidth="1"/>
+    <col min="33" max="33" width="40.1719" style="1" customWidth="1"/>
+    <col min="34" max="16384" width="16.3516" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.05" customHeight="1">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
-      <c r="C1" t="s" s="3">
+      <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="D1" t="s" s="3">
+      <c r="B1" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
-      <c r="Y1" s="4"/>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="4"/>
-      <c r="AD1" s="4"/>
-      <c r="AE1" s="4"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
+      <c r="AA1" s="3"/>
+      <c r="AB1" s="3"/>
+      <c r="AC1" s="3"/>
+      <c r="AD1" s="3"/>
+      <c r="AE1" s="3"/>
       <c r="AF1" s="4"/>
-      <c r="AG1" s="4"/>
-      <c r="AH1" s="4"/>
-      <c r="AI1" s="4"/>
+      <c r="AG1" s="5"/>
     </row>
     <row r="2" ht="21.05" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" t="s" s="5">
+      <c r="A2" t="s" s="6">
         <v>2</v>
       </c>
-      <c r="D2" t="s" s="5">
+      <c r="B2" t="s" s="6">
         <v>3</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
-      <c r="Z2" s="4"/>
-      <c r="AA2" s="4"/>
-      <c r="AB2" s="4"/>
-      <c r="AC2" s="4"/>
-      <c r="AD2" s="4"/>
-      <c r="AE2" s="4"/>
-      <c r="AF2" s="4"/>
-      <c r="AG2" s="4"/>
-      <c r="AH2" s="4"/>
-      <c r="AI2" s="4"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="3"/>
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="3"/>
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="3"/>
+      <c r="AF2" s="7"/>
+      <c r="AG2" s="8"/>
     </row>
     <row r="3" ht="21.05" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" t="s" s="5">
+      <c r="A3" t="s" s="6">
         <v>4</v>
       </c>
-      <c r="D3" t="s" s="5">
+      <c r="B3" t="s" s="6">
         <v>5</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
-      <c r="Z3" s="4"/>
-      <c r="AA3" s="4"/>
-      <c r="AB3" s="4"/>
-      <c r="AC3" s="4"/>
-      <c r="AD3" s="4"/>
-      <c r="AE3" s="4"/>
-      <c r="AF3" s="4"/>
-      <c r="AG3" s="4"/>
-      <c r="AH3" s="4"/>
-      <c r="AI3" s="4"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="8"/>
     </row>
     <row r="4" ht="19.1" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" t="s" s="5">
+      <c r="A4" t="s" s="6">
         <v>6</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="4"/>
-      <c r="Y4" s="4"/>
-      <c r="Z4" s="4"/>
-      <c r="AA4" s="4"/>
-      <c r="AB4" s="4"/>
-      <c r="AC4" s="4"/>
-      <c r="AD4" s="4"/>
-      <c r="AE4" s="4"/>
-      <c r="AF4" s="4"/>
-      <c r="AG4" s="4"/>
-      <c r="AH4" s="4"/>
-      <c r="AI4" s="4"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="7"/>
+      <c r="AG4" s="8"/>
     </row>
     <row r="5" ht="26.45" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" t="s" s="3">
+      <c r="A5" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
-      <c r="Z5" s="4"/>
-      <c r="AA5" s="4"/>
-      <c r="AB5" s="4"/>
-      <c r="AC5" s="4"/>
-      <c r="AD5" s="4"/>
-      <c r="AE5" s="4"/>
-      <c r="AF5" s="4"/>
-      <c r="AG5" s="4"/>
-      <c r="AH5" s="4"/>
-      <c r="AI5" s="4"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3"/>
+      <c r="AB5" s="3"/>
+      <c r="AC5" s="3"/>
+      <c r="AD5" s="3"/>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="10"/>
+      <c r="AG5" s="11"/>
     </row>
     <row r="6" ht="21.15" customHeight="1">
-      <c r="A6" t="s" s="8">
+      <c r="A6" t="s" s="12">
         <v>8</v>
       </c>
-      <c r="B6" t="s" s="8">
+      <c r="B6" t="s" s="13">
         <v>9</v>
       </c>
-      <c r="C6" t="s" s="9">
+      <c r="C6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="D6" t="s" s="9">
+      <c r="D6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="E6" t="s" s="9">
+      <c r="E6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="F6" t="s" s="9">
+      <c r="F6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="G6" t="s" s="9">
+      <c r="G6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="H6" t="s" s="9">
+      <c r="H6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="I6" t="s" s="9">
+      <c r="I6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="J6" t="s" s="9">
+      <c r="J6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="K6" t="s" s="9">
+      <c r="K6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="L6" t="s" s="9">
+      <c r="L6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="M6" t="s" s="9">
+      <c r="M6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="N6" t="s" s="9">
+      <c r="N6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="O6" t="s" s="9">
+      <c r="O6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="P6" t="s" s="9">
+      <c r="P6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="Q6" t="s" s="9">
+      <c r="Q6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="R6" t="s" s="9">
+      <c r="R6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="S6" t="s" s="9">
+      <c r="S6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="T6" t="s" s="9">
+      <c r="T6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="U6" t="s" s="9">
+      <c r="U6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="V6" t="s" s="9">
+      <c r="V6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="W6" t="s" s="9">
+      <c r="W6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="X6" t="s" s="9">
+      <c r="X6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="Y6" t="s" s="9">
+      <c r="Y6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="Z6" t="s" s="9">
+      <c r="Z6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="AA6" t="s" s="9">
+      <c r="AA6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="AB6" t="s" s="9">
+      <c r="AB6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="AC6" t="s" s="9">
+      <c r="AC6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="AD6" t="s" s="9">
+      <c r="AD6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="AE6" t="s" s="9">
+      <c r="AE6" t="s" s="14">
         <v>10</v>
       </c>
-      <c r="AF6" t="s" s="9">
-        <v>10</v>
-      </c>
-      <c r="AG6" t="s" s="9">
-        <v>10</v>
-      </c>
-      <c r="AH6" t="s" s="10">
+      <c r="AF6" t="s" s="15">
         <v>11</v>
       </c>
-      <c r="AI6" t="s" s="10">
+      <c r="AG6" t="s" s="15">
         <v>11</v>
       </c>
     </row>
     <row r="7" ht="12.9" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" t="s" s="11">
+      <c r="A7" s="16"/>
+      <c r="B7" s="17"/>
+      <c r="C7" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="4"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
-      <c r="Z7" s="4"/>
-      <c r="AA7" s="4"/>
-      <c r="AB7" s="4"/>
-      <c r="AC7" s="4"/>
-      <c r="AD7" s="4"/>
-      <c r="AE7" s="4"/>
-      <c r="AF7" s="4"/>
-      <c r="AG7" s="4"/>
-      <c r="AH7" t="s" s="12">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+      <c r="Y7" s="3"/>
+      <c r="Z7" s="3"/>
+      <c r="AA7" s="3"/>
+      <c r="AB7" s="3"/>
+      <c r="AC7" s="3"/>
+      <c r="AD7" s="3"/>
+      <c r="AE7" s="3"/>
+      <c r="AF7" t="s" s="19">
         <v>13</v>
       </c>
-      <c r="AI7" t="s" s="13">
+      <c r="AG7" t="s" s="20">
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="12.9" customHeight="1">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" t="s" s="11">
+    <row r="8" ht="13.55" customHeight="1">
+      <c r="A8" s="21"/>
+      <c r="B8" s="22"/>
+      <c r="C8" t="s" s="23">
         <v>14</v>
       </c>
-      <c r="D8" t="s" s="11">
+      <c r="D8" t="s" s="23">
         <v>15</v>
       </c>
-      <c r="E8" t="s" s="11">
+      <c r="E8" t="s" s="23">
         <v>16</v>
       </c>
-      <c r="F8" t="s" s="11">
+      <c r="F8" t="s" s="23">
         <v>17</v>
       </c>
-      <c r="G8" t="s" s="11">
+      <c r="G8" t="s" s="23">
         <v>18</v>
       </c>
-      <c r="H8" t="s" s="11">
+      <c r="H8" t="s" s="23">
         <v>19</v>
       </c>
-      <c r="I8" t="s" s="11">
+      <c r="I8" t="s" s="23">
         <v>20</v>
       </c>
-      <c r="J8" t="s" s="11">
+      <c r="J8" t="s" s="23">
         <v>21</v>
       </c>
-      <c r="K8" t="s" s="11">
+      <c r="K8" t="s" s="23">
         <v>22</v>
       </c>
-      <c r="L8" t="s" s="11">
+      <c r="L8" t="s" s="23">
         <v>23</v>
       </c>
-      <c r="M8" t="s" s="11">
+      <c r="M8" t="s" s="23">
         <v>24</v>
       </c>
-      <c r="N8" t="s" s="11">
+      <c r="N8" t="s" s="23">
         <v>25</v>
       </c>
-      <c r="O8" t="s" s="11">
+      <c r="O8" t="s" s="23">
         <v>26</v>
       </c>
-      <c r="P8" t="s" s="11">
+      <c r="P8" t="s" s="23">
         <v>27</v>
       </c>
-      <c r="Q8" t="s" s="11">
+      <c r="Q8" t="s" s="23">
         <v>28</v>
       </c>
-      <c r="R8" t="s" s="11">
+      <c r="R8" t="s" s="23">
         <v>29</v>
       </c>
-      <c r="S8" t="s" s="11">
+      <c r="S8" t="s" s="23">
         <v>30</v>
       </c>
-      <c r="T8" t="s" s="11">
+      <c r="T8" t="s" s="23">
         <v>31</v>
       </c>
-      <c r="U8" t="s" s="11">
+      <c r="U8" t="s" s="23">
         <v>32</v>
       </c>
-      <c r="V8" t="s" s="11">
+      <c r="V8" t="s" s="23">
         <v>33</v>
       </c>
-      <c r="W8" t="s" s="11">
+      <c r="W8" t="s" s="23">
         <v>34</v>
       </c>
-      <c r="X8" t="s" s="11">
+      <c r="X8" t="s" s="23">
         <v>35</v>
       </c>
-      <c r="Y8" t="s" s="11">
+      <c r="Y8" t="s" s="23">
         <v>36</v>
       </c>
-      <c r="Z8" t="s" s="11">
+      <c r="Z8" t="s" s="23">
         <v>37</v>
       </c>
-      <c r="AA8" t="s" s="11">
+      <c r="AA8" t="s" s="23">
         <v>38</v>
       </c>
-      <c r="AB8" t="s" s="11">
+      <c r="AB8" t="s" s="23">
         <v>39</v>
       </c>
-      <c r="AC8" t="s" s="11">
+      <c r="AC8" t="s" s="23">
         <v>40</v>
       </c>
-      <c r="AD8" t="s" s="11">
+      <c r="AD8" t="s" s="23">
         <v>41</v>
       </c>
-      <c r="AE8" t="s" s="11">
+      <c r="AE8" t="s" s="23">
         <v>42</v>
       </c>
-      <c r="AF8" t="s" s="11">
+      <c r="AF8" t="s" s="24">
         <v>43</v>
       </c>
-      <c r="AG8" t="s" s="11">
+      <c r="AG8" t="s" s="24">
         <v>44</v>
-      </c>
-      <c r="AH8" t="s" s="14">
-        <v>45</v>
-      </c>
-      <c r="AI8" t="s" s="14">
-        <v>46</v>
       </c>
     </row>
     <row r="9" ht="12.9" customHeight="1" hidden="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" t="s" s="15">
+      <c r="A9" s="21"/>
+      <c r="B9" s="25"/>
+      <c r="C9" t="s" s="26">
+        <v>45</v>
+      </c>
+      <c r="D9" t="s" s="26">
+        <v>46</v>
+      </c>
+      <c r="E9" t="s" s="26">
         <v>47</v>
       </c>
-      <c r="D9" t="s" s="15">
+      <c r="F9" t="s" s="26">
         <v>48</v>
       </c>
-      <c r="E9" t="s" s="15">
+      <c r="G9" t="s" s="26">
         <v>49</v>
       </c>
-      <c r="F9" t="s" s="15">
+      <c r="H9" t="s" s="26">
         <v>50</v>
       </c>
-      <c r="G9" t="s" s="15">
+      <c r="I9" t="s" s="23">
         <v>51</v>
       </c>
-      <c r="H9" t="s" s="15">
+      <c r="J9" t="s" s="23">
         <v>52</v>
       </c>
-      <c r="I9" t="s" s="15">
+      <c r="K9" t="s" s="23">
         <v>53</v>
       </c>
-      <c r="J9" t="s" s="15">
+      <c r="L9" t="s" s="23">
         <v>54</v>
       </c>
-      <c r="K9" t="s" s="11">
+      <c r="M9" t="s" s="23">
         <v>55</v>
       </c>
-      <c r="L9" t="s" s="11">
+      <c r="N9" t="s" s="23">
         <v>56</v>
       </c>
-      <c r="M9" t="s" s="11">
+      <c r="O9" t="s" s="23">
         <v>57</v>
       </c>
-      <c r="N9" t="s" s="11">
+      <c r="P9" t="s" s="23">
         <v>58</v>
       </c>
-      <c r="O9" t="s" s="11">
+      <c r="Q9" t="s" s="23">
         <v>59</v>
       </c>
-      <c r="P9" t="s" s="11">
+      <c r="R9" t="s" s="23">
         <v>60</v>
       </c>
-      <c r="Q9" t="s" s="11">
+      <c r="S9" t="s" s="23">
         <v>61</v>
       </c>
-      <c r="R9" t="s" s="11">
+      <c r="T9" t="s" s="23">
         <v>62</v>
       </c>
-      <c r="S9" t="s" s="11">
+      <c r="U9" t="s" s="23">
         <v>63</v>
       </c>
-      <c r="T9" t="s" s="11">
+      <c r="V9" t="s" s="23">
         <v>64</v>
       </c>
-      <c r="U9" t="s" s="11">
+      <c r="W9" t="s" s="23">
         <v>65</v>
       </c>
-      <c r="V9" t="s" s="11">
+      <c r="X9" t="s" s="23">
         <v>66</v>
       </c>
-      <c r="W9" t="s" s="11">
+      <c r="Y9" t="s" s="23">
         <v>67</v>
       </c>
-      <c r="X9" t="s" s="11">
+      <c r="Z9" t="s" s="23">
         <v>68</v>
       </c>
-      <c r="Y9" t="s" s="11">
+      <c r="AA9" t="s" s="23">
         <v>69</v>
       </c>
-      <c r="Z9" t="s" s="11">
+      <c r="AB9" t="s" s="23">
         <v>70</v>
       </c>
-      <c r="AA9" t="s" s="11">
+      <c r="AC9" t="s" s="23">
         <v>71</v>
       </c>
-      <c r="AB9" t="s" s="11">
+      <c r="AD9" t="s" s="23">
         <v>72</v>
       </c>
-      <c r="AC9" t="s" s="11">
+      <c r="AE9" t="s" s="23">
         <v>73</v>
       </c>
-      <c r="AD9" t="s" s="11">
-        <v>74</v>
-      </c>
-      <c r="AE9" t="s" s="11">
-        <v>75</v>
-      </c>
-      <c r="AF9" t="s" s="11">
-        <v>76</v>
-      </c>
-      <c r="AG9" t="s" s="11">
-        <v>77</v>
-      </c>
-      <c r="AH9" s="14"/>
-      <c r="AI9" s="14"/>
+      <c r="AF9" s="24"/>
+      <c r="AG9" s="24"/>
     </row>
     <row r="10" ht="12.9" customHeight="1" hidden="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" t="s" s="16">
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" t="s" s="27">
+        <v>74</v>
+      </c>
+      <c r="D10" t="s" s="27">
+        <v>75</v>
+      </c>
+      <c r="E10" t="s" s="27">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s" s="27">
+        <v>77</v>
+      </c>
+      <c r="G10" t="s" s="27">
         <v>78</v>
       </c>
-      <c r="F10" t="s" s="16">
+      <c r="H10" t="s" s="27">
         <v>79</v>
       </c>
-      <c r="G10" t="s" s="16">
+      <c r="I10" t="s" s="27">
         <v>80</v>
       </c>
-      <c r="H10" t="s" s="16">
+      <c r="J10" t="s" s="27">
         <v>81</v>
       </c>
-      <c r="I10" t="s" s="16">
+      <c r="K10" t="s" s="27">
         <v>82</v>
       </c>
-      <c r="J10" t="s" s="16">
+      <c r="L10" t="s" s="27">
         <v>83</v>
       </c>
-      <c r="K10" t="s" s="16">
+      <c r="M10" t="s" s="27">
         <v>84</v>
       </c>
-      <c r="L10" t="s" s="16">
+      <c r="N10" t="s" s="27">
         <v>85</v>
       </c>
-      <c r="M10" t="s" s="16">
+      <c r="O10" t="s" s="27">
         <v>86</v>
       </c>
-      <c r="N10" t="s" s="16">
+      <c r="P10" t="s" s="27">
         <v>87</v>
       </c>
-      <c r="O10" t="s" s="16">
+      <c r="Q10" t="s" s="27">
         <v>88</v>
       </c>
-      <c r="P10" t="s" s="16">
+      <c r="R10" t="s" s="27">
         <v>89</v>
       </c>
-      <c r="Q10" t="s" s="16">
+      <c r="S10" t="s" s="27">
         <v>90</v>
       </c>
-      <c r="R10" t="s" s="16">
+      <c r="T10" t="s" s="27">
         <v>91</v>
       </c>
-      <c r="S10" t="s" s="16">
+      <c r="U10" t="s" s="27">
         <v>92</v>
       </c>
-      <c r="T10" t="s" s="16">
+      <c r="V10" t="s" s="27">
         <v>93</v>
       </c>
-      <c r="U10" t="s" s="16">
+      <c r="W10" t="s" s="27">
         <v>94</v>
       </c>
-      <c r="V10" t="s" s="16">
+      <c r="X10" t="s" s="27">
         <v>95</v>
       </c>
-      <c r="W10" t="s" s="16">
+      <c r="Y10" t="s" s="27">
         <v>96</v>
       </c>
-      <c r="X10" t="s" s="16">
+      <c r="Z10" t="s" s="27">
         <v>97</v>
       </c>
-      <c r="Y10" t="s" s="16">
+      <c r="AA10" t="s" s="27">
         <v>98</v>
       </c>
-      <c r="Z10" t="s" s="16">
+      <c r="AB10" t="s" s="27">
         <v>99</v>
       </c>
-      <c r="AA10" t="s" s="16">
+      <c r="AC10" t="s" s="27">
         <v>100</v>
       </c>
-      <c r="AB10" t="s" s="16">
+      <c r="AD10" t="s" s="27">
         <v>101</v>
       </c>
-      <c r="AC10" t="s" s="16">
+      <c r="AE10" t="s" s="27">
         <v>102</v>
       </c>
-      <c r="AD10" t="s" s="16">
-        <v>103</v>
-      </c>
-      <c r="AE10" t="s" s="16">
-        <v>104</v>
-      </c>
-      <c r="AF10" t="s" s="16">
-        <v>105</v>
-      </c>
-      <c r="AG10" t="s" s="16">
-        <v>106</v>
-      </c>
-      <c r="AH10" s="14"/>
-      <c r="AI10" s="14"/>
+      <c r="AF10" s="24"/>
+      <c r="AG10" s="24"/>
     </row>
     <row r="11" ht="18.95" customHeight="1">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" t="s" s="17">
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" t="s" s="29">
+        <v>103</v>
+      </c>
+      <c r="D11" t="s" s="30">
+        <v>104</v>
+      </c>
+      <c r="E11" t="s" s="30">
+        <v>105</v>
+      </c>
+      <c r="F11" t="s" s="30">
+        <v>106</v>
+      </c>
+      <c r="G11" t="s" s="30">
         <v>107</v>
       </c>
-      <c r="D11" t="s" s="18">
+      <c r="H11" t="s" s="30">
         <v>108</v>
       </c>
-      <c r="E11" t="s" s="18">
+      <c r="I11" t="s" s="30">
         <v>109</v>
       </c>
-      <c r="F11" t="s" s="18">
+      <c r="J11" t="s" s="30">
         <v>110</v>
       </c>
-      <c r="G11" t="s" s="18">
+      <c r="K11" t="s" s="30">
         <v>111</v>
       </c>
-      <c r="H11" t="s" s="18">
+      <c r="L11" t="s" s="30">
         <v>112</v>
       </c>
-      <c r="I11" t="s" s="18">
+      <c r="M11" t="s" s="30">
         <v>113</v>
       </c>
-      <c r="J11" t="s" s="18">
+      <c r="N11" t="s" s="30">
         <v>114</v>
       </c>
-      <c r="K11" t="s" s="18">
+      <c r="O11" t="s" s="30">
         <v>115</v>
       </c>
-      <c r="L11" t="s" s="18">
+      <c r="P11" t="s" s="30">
         <v>116</v>
       </c>
-      <c r="M11" t="s" s="18">
+      <c r="Q11" t="s" s="30">
         <v>117</v>
       </c>
-      <c r="N11" t="s" s="18">
+      <c r="R11" t="s" s="30">
         <v>118</v>
       </c>
-      <c r="O11" t="s" s="18">
+      <c r="S11" t="s" s="30">
         <v>119</v>
       </c>
-      <c r="P11" t="s" s="18">
+      <c r="T11" t="s" s="30">
         <v>120</v>
       </c>
-      <c r="Q11" t="s" s="18">
+      <c r="U11" t="s" s="30">
         <v>121</v>
       </c>
-      <c r="R11" t="s" s="18">
+      <c r="V11" t="s" s="30">
         <v>122</v>
       </c>
-      <c r="S11" t="s" s="18">
+      <c r="W11" t="s" s="30">
         <v>123</v>
       </c>
-      <c r="T11" t="s" s="18">
+      <c r="X11" t="s" s="30">
         <v>124</v>
       </c>
-      <c r="U11" t="s" s="18">
+      <c r="Y11" t="s" s="30">
         <v>125</v>
       </c>
-      <c r="V11" t="s" s="18">
+      <c r="Z11" t="s" s="30">
         <v>126</v>
       </c>
-      <c r="W11" t="s" s="18">
+      <c r="AA11" t="s" s="30">
         <v>127</v>
       </c>
-      <c r="X11" t="s" s="18">
+      <c r="AB11" t="s" s="30">
         <v>128</v>
       </c>
-      <c r="Y11" t="s" s="18">
+      <c r="AC11" t="s" s="30">
         <v>129</v>
       </c>
-      <c r="Z11" t="s" s="18">
+      <c r="AD11" t="s" s="30">
         <v>130</v>
       </c>
-      <c r="AA11" t="s" s="18">
+      <c r="AE11" t="s" s="30">
         <v>131</v>
       </c>
-      <c r="AB11" t="s" s="18">
+      <c r="AF11" t="s" s="30">
         <v>132</v>
       </c>
-      <c r="AC11" t="s" s="18">
+      <c r="AG11" t="s" s="31">
         <v>133</v>
-      </c>
-      <c r="AD11" t="s" s="18">
-        <v>134</v>
-      </c>
-      <c r="AE11" t="s" s="18">
-        <v>135</v>
-      </c>
-      <c r="AF11" t="s" s="18">
-        <v>136</v>
-      </c>
-      <c r="AG11" t="s" s="18">
-        <v>137</v>
-      </c>
-      <c r="AH11" t="s" s="18">
-        <v>138</v>
-      </c>
-      <c r="AI11" t="s" s="19">
-        <v>139</v>
       </c>
     </row>
     <row r="12" ht="12.9" customHeight="1">
-      <c r="A12" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="B12" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="C12" t="s" s="20">
-        <v>142</v>
-      </c>
-      <c r="D12" t="s" s="20">
-        <v>143</v>
-      </c>
-      <c r="E12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="F12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="G12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="H12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="I12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="J12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="K12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="L12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="M12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="N12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="O12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="P12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Q12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="R12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="S12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="T12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="U12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="V12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="W12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="X12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Y12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Z12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AA12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AB12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AC12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AD12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AE12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AF12" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AG12" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AH12" t="s" s="20">
-        <v>146</v>
-      </c>
-      <c r="AI12" t="s" s="20">
-        <v>147</v>
+      <c r="A12" t="s" s="28">
+        <v>134</v>
+      </c>
+      <c r="B12" t="s" s="28">
+        <v>135</v>
+      </c>
+      <c r="C12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="D12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="E12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="F12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="G12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="H12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="I12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="J12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="K12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="L12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="M12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="N12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="O12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="P12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Q12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="R12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="S12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="T12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="U12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="V12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="W12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="X12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Y12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Z12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AA12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AB12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AC12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AD12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AE12" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AF12" t="s" s="32">
+        <v>137</v>
+      </c>
+      <c r="AG12" t="s" s="32">
+        <v>138</v>
       </c>
     </row>
     <row r="13" ht="12.9" customHeight="1">
-      <c r="A13" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="B13" t="s" s="2">
+      <c r="A13" t="s" s="28">
+        <v>139</v>
+      </c>
+      <c r="B13" t="s" s="28">
+        <v>140</v>
+      </c>
+      <c r="C13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="D13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="E13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="F13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="G13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="H13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="I13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="J13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="K13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="L13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="M13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="N13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="O13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="P13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Q13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="R13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="S13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="T13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="U13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="V13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="W13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="X13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Y13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Z13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AA13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AB13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AC13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AD13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AE13" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AF13" t="s" s="32">
+        <v>137</v>
+      </c>
+      <c r="AG13" t="s" s="32">
         <v>141</v>
-      </c>
-      <c r="C13" t="s" s="20">
-        <v>142</v>
-      </c>
-      <c r="D13" t="s" s="20">
-        <v>143</v>
-      </c>
-      <c r="E13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="F13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="G13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="H13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="I13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="J13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="K13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="L13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="M13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="N13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="O13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="P13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Q13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="R13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="S13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="T13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="U13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="V13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="W13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="X13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Y13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Z13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AA13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AB13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AC13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AD13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AE13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AF13" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AG13" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AH13" t="s" s="20">
-        <v>146</v>
-      </c>
-      <c r="AI13" t="s" s="20">
-        <v>147</v>
       </c>
     </row>
     <row r="14" ht="12.9" customHeight="1">
-      <c r="A14" t="s" s="2">
-        <v>149</v>
-      </c>
-      <c r="B14" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="C14" t="s" s="20">
+      <c r="A14" t="s" s="28">
         <v>142</v>
       </c>
-      <c r="D14" t="s" s="20">
+      <c r="B14" t="s" s="28">
         <v>143</v>
       </c>
-      <c r="E14" t="s" s="20">
+      <c r="C14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="D14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="E14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="F14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="G14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="H14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="I14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="J14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="K14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="L14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="M14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="N14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="O14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="P14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Q14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="R14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="S14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="T14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="U14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="V14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="W14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="X14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Y14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Z14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AA14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AB14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AC14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AD14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AE14" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AF14" t="s" s="32">
+        <v>137</v>
+      </c>
+      <c r="AG14" t="s" s="32">
         <v>144</v>
-      </c>
-      <c r="F14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="G14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="H14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="I14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="J14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="K14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="L14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="M14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="N14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="O14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="P14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Q14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="R14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="S14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="T14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="U14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="V14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="W14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="X14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Y14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="Z14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AA14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AB14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AC14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AD14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AE14" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AF14" t="s" s="20">
-        <v>144</v>
-      </c>
-      <c r="AG14" t="s" s="20">
-        <v>145</v>
-      </c>
-      <c r="AH14" t="s" s="20">
-        <v>146</v>
-      </c>
-      <c r="AI14" t="s" s="20">
-        <v>147</v>
       </c>
     </row>
     <row r="15" ht="12.9" customHeight="1">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-      <c r="M15" s="20"/>
-      <c r="N15" s="20"/>
-      <c r="O15" s="20"/>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="20"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="20"/>
-      <c r="T15" s="20"/>
-      <c r="U15" s="20"/>
-      <c r="V15" s="20"/>
-      <c r="W15" s="20"/>
-      <c r="X15" s="20"/>
-      <c r="Y15" s="20"/>
-      <c r="Z15" s="20"/>
-      <c r="AA15" s="20"/>
-      <c r="AB15" s="20"/>
-      <c r="AC15" s="20"/>
-      <c r="AD15" s="20"/>
-      <c r="AE15" s="20"/>
-      <c r="AF15" s="20"/>
-      <c r="AG15" s="20"/>
-      <c r="AH15" s="20"/>
-      <c r="AI15" s="20"/>
+      <c r="A15" t="s" s="28">
+        <v>145</v>
+      </c>
+      <c r="B15" t="s" s="28">
+        <v>146</v>
+      </c>
+      <c r="C15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="D15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="E15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="F15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="G15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="H15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="I15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="J15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="K15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="L15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="M15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="N15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="O15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="P15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Q15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="R15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="S15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="T15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="U15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="V15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="W15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="X15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Y15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="Z15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AA15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AB15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AC15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AD15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AE15" t="s" s="32">
+        <v>136</v>
+      </c>
+      <c r="AF15" t="s" s="32">
+        <v>137</v>
+      </c>
+      <c r="AG15" t="s" s="32">
+        <v>147</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="C7:AG7"/>
-    <mergeCell ref="D1:AI1"/>
-    <mergeCell ref="D2:AI2"/>
-    <mergeCell ref="D3:AI3"/>
-    <mergeCell ref="C5:AI5"/>
-    <mergeCell ref="D4:AI4"/>
+    <mergeCell ref="C7:AE7"/>
+    <mergeCell ref="A5:AG5"/>
+    <mergeCell ref="B4:AG4"/>
+    <mergeCell ref="B3:AG3"/>
+    <mergeCell ref="B2:AG2"/>
+    <mergeCell ref="B1:AG1"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
backup-restore + rule cell modification using dashboard
</commit_message>
<xml_diff>
--- a/backup/rules_2.xlsx
+++ b/backup/rules_2.xlsx
@@ -418,7 +418,7 @@
     <t>activeToFreezeR</t>
   </si>
   <si>
-    <t>"activeToFreeze"</t>
+    <t>activeToFreeze</t>
   </si>
   <si>
     <t>N</t>
@@ -433,7 +433,7 @@
     <t>activeToSelllingOnlyR</t>
   </si>
   <si>
-    <t>"activeToSellingOnly"</t>
+    <t>activeToSellingOnly</t>
   </si>
   <si>
     <t>SELLING ONLY</t>
@@ -442,7 +442,7 @@
     <t>activeToInactiveR</t>
   </si>
   <si>
-    <t>"activeToInactive"</t>
+    <t>activeToInactive</t>
   </si>
   <si>
     <t>INACTIVE</t>
@@ -451,7 +451,7 @@
     <t>activeToBuyingOnlyR</t>
   </si>
   <si>
-    <t>"activeToBuyingOnly"</t>
+    <t>activeToBuyingOnly</t>
   </si>
   <si>
     <t>BUYING ONLY</t>
@@ -586,7 +586,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -773,11 +773,44 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
         <color indexed="11"/>
       </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="11"/>
       </bottom>
@@ -789,7 +822,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -871,16 +904,25 @@
     <xf numFmtId="49" fontId="0" fillId="11" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="12" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="13" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="13" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="13" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="13" borderId="18" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="13" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -2411,7 +2453,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" ht="12.9" customHeight="1" hidden="1">
+    <row r="9" ht="12.9" customHeight="1">
       <c r="A9" s="21"/>
       <c r="B9" s="25"/>
       <c r="C9" t="s" s="26">
@@ -2501,600 +2543,600 @@
       <c r="AE9" t="s" s="23">
         <v>73</v>
       </c>
-      <c r="AF9" s="24"/>
+      <c r="AF9" s="27"/>
       <c r="AG9" s="24"/>
     </row>
-    <row r="10" ht="12.9" customHeight="1" hidden="1">
+    <row r="10" ht="12.9" customHeight="1">
       <c r="A10" s="21"/>
       <c r="B10" s="21"/>
-      <c r="C10" t="s" s="27">
+      <c r="C10" t="s" s="28">
         <v>74</v>
       </c>
-      <c r="D10" t="s" s="27">
+      <c r="D10" t="s" s="28">
         <v>75</v>
       </c>
-      <c r="E10" t="s" s="27">
+      <c r="E10" t="s" s="28">
         <v>76</v>
       </c>
-      <c r="F10" t="s" s="27">
+      <c r="F10" t="s" s="28">
         <v>77</v>
       </c>
-      <c r="G10" t="s" s="27">
+      <c r="G10" t="s" s="28">
         <v>78</v>
       </c>
-      <c r="H10" t="s" s="27">
+      <c r="H10" t="s" s="28">
         <v>79</v>
       </c>
-      <c r="I10" t="s" s="27">
+      <c r="I10" t="s" s="28">
         <v>80</v>
       </c>
-      <c r="J10" t="s" s="27">
+      <c r="J10" t="s" s="28">
         <v>81</v>
       </c>
-      <c r="K10" t="s" s="27">
+      <c r="K10" t="s" s="28">
         <v>82</v>
       </c>
-      <c r="L10" t="s" s="27">
+      <c r="L10" t="s" s="28">
         <v>83</v>
       </c>
-      <c r="M10" t="s" s="27">
+      <c r="M10" t="s" s="28">
         <v>84</v>
       </c>
-      <c r="N10" t="s" s="27">
+      <c r="N10" t="s" s="28">
         <v>85</v>
       </c>
-      <c r="O10" t="s" s="27">
+      <c r="O10" t="s" s="28">
         <v>86</v>
       </c>
-      <c r="P10" t="s" s="27">
+      <c r="P10" t="s" s="28">
         <v>87</v>
       </c>
-      <c r="Q10" t="s" s="27">
+      <c r="Q10" t="s" s="28">
         <v>88</v>
       </c>
-      <c r="R10" t="s" s="27">
+      <c r="R10" t="s" s="28">
         <v>89</v>
       </c>
-      <c r="S10" t="s" s="27">
+      <c r="S10" t="s" s="28">
         <v>90</v>
       </c>
-      <c r="T10" t="s" s="27">
+      <c r="T10" t="s" s="28">
         <v>91</v>
       </c>
-      <c r="U10" t="s" s="27">
+      <c r="U10" t="s" s="28">
         <v>92</v>
       </c>
-      <c r="V10" t="s" s="27">
+      <c r="V10" t="s" s="28">
         <v>93</v>
       </c>
-      <c r="W10" t="s" s="27">
+      <c r="W10" t="s" s="28">
         <v>94</v>
       </c>
-      <c r="X10" t="s" s="27">
+      <c r="X10" t="s" s="28">
         <v>95</v>
       </c>
-      <c r="Y10" t="s" s="27">
+      <c r="Y10" t="s" s="28">
         <v>96</v>
       </c>
-      <c r="Z10" t="s" s="27">
+      <c r="Z10" t="s" s="28">
         <v>97</v>
       </c>
-      <c r="AA10" t="s" s="27">
+      <c r="AA10" t="s" s="28">
         <v>98</v>
       </c>
-      <c r="AB10" t="s" s="27">
+      <c r="AB10" t="s" s="28">
         <v>99</v>
       </c>
-      <c r="AC10" t="s" s="27">
+      <c r="AC10" t="s" s="28">
         <v>100</v>
       </c>
-      <c r="AD10" t="s" s="27">
+      <c r="AD10" t="s" s="28">
         <v>101</v>
       </c>
-      <c r="AE10" t="s" s="27">
+      <c r="AE10" t="s" s="28">
         <v>102</v>
       </c>
-      <c r="AF10" s="24"/>
+      <c r="AF10" s="29"/>
       <c r="AG10" s="24"/>
     </row>
     <row r="11" ht="18.95" customHeight="1">
-      <c r="A11" s="28"/>
-      <c r="B11" s="28"/>
-      <c r="C11" t="s" s="29">
+      <c r="A11" s="30"/>
+      <c r="B11" s="30"/>
+      <c r="C11" t="s" s="31">
         <v>103</v>
       </c>
-      <c r="D11" t="s" s="30">
+      <c r="D11" t="s" s="32">
         <v>104</v>
       </c>
-      <c r="E11" t="s" s="30">
+      <c r="E11" t="s" s="32">
         <v>105</v>
       </c>
-      <c r="F11" t="s" s="30">
+      <c r="F11" t="s" s="32">
         <v>106</v>
       </c>
-      <c r="G11" t="s" s="30">
+      <c r="G11" t="s" s="32">
         <v>107</v>
       </c>
-      <c r="H11" t="s" s="30">
+      <c r="H11" t="s" s="32">
         <v>108</v>
       </c>
-      <c r="I11" t="s" s="30">
+      <c r="I11" t="s" s="32">
         <v>109</v>
       </c>
-      <c r="J11" t="s" s="30">
+      <c r="J11" t="s" s="32">
         <v>110</v>
       </c>
-      <c r="K11" t="s" s="30">
+      <c r="K11" t="s" s="32">
         <v>111</v>
       </c>
-      <c r="L11" t="s" s="30">
+      <c r="L11" t="s" s="32">
         <v>112</v>
       </c>
-      <c r="M11" t="s" s="30">
+      <c r="M11" t="s" s="32">
         <v>113</v>
       </c>
-      <c r="N11" t="s" s="30">
+      <c r="N11" t="s" s="32">
         <v>114</v>
       </c>
-      <c r="O11" t="s" s="30">
+      <c r="O11" t="s" s="32">
         <v>115</v>
       </c>
-      <c r="P11" t="s" s="30">
+      <c r="P11" t="s" s="32">
         <v>116</v>
       </c>
-      <c r="Q11" t="s" s="30">
+      <c r="Q11" t="s" s="32">
         <v>117</v>
       </c>
-      <c r="R11" t="s" s="30">
+      <c r="R11" t="s" s="32">
         <v>118</v>
       </c>
-      <c r="S11" t="s" s="30">
+      <c r="S11" t="s" s="32">
         <v>119</v>
       </c>
-      <c r="T11" t="s" s="30">
+      <c r="T11" t="s" s="32">
         <v>120</v>
       </c>
-      <c r="U11" t="s" s="30">
+      <c r="U11" t="s" s="32">
         <v>121</v>
       </c>
-      <c r="V11" t="s" s="30">
+      <c r="V11" t="s" s="32">
         <v>122</v>
       </c>
-      <c r="W11" t="s" s="30">
+      <c r="W11" t="s" s="32">
         <v>123</v>
       </c>
-      <c r="X11" t="s" s="30">
+      <c r="X11" t="s" s="32">
         <v>124</v>
       </c>
-      <c r="Y11" t="s" s="30">
+      <c r="Y11" t="s" s="32">
         <v>125</v>
       </c>
-      <c r="Z11" t="s" s="30">
+      <c r="Z11" t="s" s="32">
         <v>126</v>
       </c>
-      <c r="AA11" t="s" s="30">
+      <c r="AA11" t="s" s="32">
         <v>127</v>
       </c>
-      <c r="AB11" t="s" s="30">
+      <c r="AB11" t="s" s="32">
         <v>128</v>
       </c>
-      <c r="AC11" t="s" s="30">
+      <c r="AC11" t="s" s="32">
         <v>129</v>
       </c>
-      <c r="AD11" t="s" s="30">
+      <c r="AD11" t="s" s="32">
         <v>130</v>
       </c>
-      <c r="AE11" t="s" s="30">
+      <c r="AE11" t="s" s="32">
         <v>131</v>
       </c>
-      <c r="AF11" t="s" s="30">
+      <c r="AF11" t="s" s="33">
         <v>132</v>
       </c>
-      <c r="AG11" t="s" s="31">
+      <c r="AG11" t="s" s="34">
         <v>133</v>
       </c>
     </row>
     <row r="12" ht="12.9" customHeight="1">
-      <c r="A12" t="s" s="28">
+      <c r="A12" t="s" s="30">
         <v>134</v>
       </c>
-      <c r="B12" t="s" s="28">
+      <c r="B12" t="s" s="30">
         <v>135</v>
       </c>
-      <c r="C12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="D12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="E12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="F12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="G12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="H12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="I12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="J12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="K12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="L12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="M12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="N12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="O12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="P12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Q12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="R12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="S12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="T12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="U12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="V12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="W12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="X12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Y12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Z12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AA12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AB12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AC12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AD12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AE12" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AF12" t="s" s="32">
+      <c r="C12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="D12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="E12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="F12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="G12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="H12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="I12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="J12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="K12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="L12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="M12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="N12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="O12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="P12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Q12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="R12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="S12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="T12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="U12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="V12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="W12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="X12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Y12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Z12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AA12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AB12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AC12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AD12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AE12" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AF12" t="s" s="35">
         <v>137</v>
       </c>
-      <c r="AG12" t="s" s="32">
+      <c r="AG12" t="s" s="35">
         <v>138</v>
       </c>
     </row>
     <row r="13" ht="12.9" customHeight="1">
-      <c r="A13" t="s" s="28">
+      <c r="A13" t="s" s="30">
         <v>139</v>
       </c>
-      <c r="B13" t="s" s="28">
+      <c r="B13" t="s" s="30">
         <v>140</v>
       </c>
-      <c r="C13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="D13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="E13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="F13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="G13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="H13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="I13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="J13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="K13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="L13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="M13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="N13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="O13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="P13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Q13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="R13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="S13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="T13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="U13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="V13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="W13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="X13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Y13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Z13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AA13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AB13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AC13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AD13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AE13" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AF13" t="s" s="32">
+      <c r="C13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="D13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="E13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="F13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="G13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="H13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="I13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="J13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="K13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="L13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="M13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="N13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="O13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="P13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Q13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="R13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="S13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="T13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="U13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="V13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="W13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="X13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Y13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Z13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AA13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AB13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AC13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AD13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AE13" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AF13" t="s" s="35">
         <v>137</v>
       </c>
-      <c r="AG13" t="s" s="32">
+      <c r="AG13" t="s" s="35">
         <v>141</v>
       </c>
     </row>
     <row r="14" ht="12.9" customHeight="1">
-      <c r="A14" t="s" s="28">
+      <c r="A14" t="s" s="30">
         <v>142</v>
       </c>
-      <c r="B14" t="s" s="28">
+      <c r="B14" t="s" s="30">
         <v>143</v>
       </c>
-      <c r="C14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="D14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="E14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="F14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="G14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="H14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="I14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="J14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="K14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="L14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="M14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="N14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="O14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="P14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Q14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="R14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="S14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="T14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="U14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="V14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="W14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="X14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Y14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Z14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AA14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AB14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AC14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AD14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AE14" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AF14" t="s" s="32">
+      <c r="C14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="D14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="E14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="F14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="G14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="H14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="I14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="J14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="K14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="L14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="M14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="N14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="O14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="P14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Q14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="R14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="S14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="T14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="U14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="V14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="W14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="X14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Y14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Z14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AA14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AB14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AC14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AD14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AE14" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AF14" t="s" s="35">
         <v>137</v>
       </c>
-      <c r="AG14" t="s" s="32">
+      <c r="AG14" t="s" s="35">
         <v>144</v>
       </c>
     </row>
     <row r="15" ht="12.9" customHeight="1">
-      <c r="A15" t="s" s="28">
+      <c r="A15" t="s" s="30">
         <v>145</v>
       </c>
-      <c r="B15" t="s" s="28">
+      <c r="B15" t="s" s="30">
         <v>146</v>
       </c>
-      <c r="C15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="D15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="E15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="F15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="G15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="H15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="I15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="J15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="K15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="L15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="M15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="N15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="O15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="P15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Q15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="R15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="S15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="T15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="U15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="V15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="W15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="X15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Y15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="Z15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AA15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AB15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AC15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AD15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AE15" t="s" s="32">
-        <v>136</v>
-      </c>
-      <c r="AF15" t="s" s="32">
+      <c r="C15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="D15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="E15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="F15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="G15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="H15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="I15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="J15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="K15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="L15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="M15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="N15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="O15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="P15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Q15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="R15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="S15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="T15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="U15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="V15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="W15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="X15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Y15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="Z15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AA15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AB15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AC15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AD15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AE15" t="s" s="35">
+        <v>136</v>
+      </c>
+      <c r="AF15" t="s" s="35">
         <v>137</v>
       </c>
-      <c r="AG15" t="s" s="32">
+      <c r="AG15" t="s" s="35">
         <v>147</v>
       </c>
     </row>

</xml_diff>